<commit_message>
Add Codex-compatible test design workflow
</commit_message>
<xml_diff>
--- a/docs/test-design/codebuddy-test-design-template.xlsx
+++ b/docs/test-design/codebuddy-test-design-template.xlsx
@@ -2,13 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试设计总览" sheetId="1" r:id="Rfeb579c8d1574576"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求用户故事拆解" sheetId="2" r:id="Rcdf73bfec6914f41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试场景矩阵" sheetId="3" r:id="Ra173509e40254319"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="功能测试用例" sheetId="4" r:id="R762e10c6e1884369"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="性能测试设计" sheetId="5" r:id="Re4f603de8dbf4056"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="风险与待确认问题" sheetId="6" r:id="R20e70dcbb8ba4f7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="自动化建议" sheetId="7" r:id="R63961be21da74392"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试设计总览" sheetId="1" r:id="R9aa33bee0d574f17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求用户故事拆解" sheetId="2" r:id="R18f5be85b0144db7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试场景矩阵" sheetId="3" r:id="R1a4ee64b440c4215"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="功能测试用例" sheetId="4" r:id="R02a802871df5433f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="性能测试设计" sheetId="5" r:id="Rb4636ab274a240e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="风险与待确认问题" sheetId="6" r:id="Rd0ebf766eafd4cf2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="自动化建议" sheetId="7" r:id="R889d5606f2f34f02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面元素覆盖清单" sheetId="8" r:id="Rb1671cdb3346494e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -36,12 +37,22 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E79"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E79"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -69,7 +80,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="11">
+  <x:cellXfs count="23">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -93,11 +104,66 @@
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PageElementCoverageTable" displayName="PageElementCoverageTable" ref="A1:O3" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="15">
+    <x:tableColumn id="1" name="元素 ID"/>
+    <x:tableColumn id="2" name="Story ID/需求 ID"/>
+    <x:tableColumn id="3" name="页面/入口"/>
+    <x:tableColumn id="4" name="页面 URL/菜单路径"/>
+    <x:tableColumn id="5" name="元素名称/文案"/>
+    <x:tableColumn id="6" name="元素类型"/>
+    <x:tableColumn id="7" name="交互方式"/>
+    <x:tableColumn id="8" name="前置状态/权限"/>
+    <x:tableColumn id="9" name="预期行为"/>
+    <x:tableColumn id="10" name="业务依据/规则来源"/>
+    <x:tableColumn id="11" name="覆盖用例 ID"/>
+    <x:tableColumn id="12" name="覆盖状态"/>
+    <x:tableColumn id="13" name="发现方式"/>
+    <x:tableColumn id="14" name="素材来源"/>
+    <x:tableColumn id="15" name="待确认问题/备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1264,4 +1330,209 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="32" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="32" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="32" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="20" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="20" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="34" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="22" t="str">
+        <x:v>元素 ID</x:v>
+      </x:c>
+      <x:c r="B1" s="22" t="str">
+        <x:v>Story ID/需求 ID</x:v>
+      </x:c>
+      <x:c r="C1" s="22" t="str">
+        <x:v>页面/入口</x:v>
+      </x:c>
+      <x:c r="D1" s="22" t="str">
+        <x:v>页面 URL/菜单路径</x:v>
+      </x:c>
+      <x:c r="E1" s="22" t="str">
+        <x:v>元素名称/文案</x:v>
+      </x:c>
+      <x:c r="F1" s="22" t="str">
+        <x:v>元素类型</x:v>
+      </x:c>
+      <x:c r="G1" s="22" t="str">
+        <x:v>交互方式</x:v>
+      </x:c>
+      <x:c r="H1" s="22" t="str">
+        <x:v>前置状态/权限</x:v>
+      </x:c>
+      <x:c r="I1" s="22" t="str">
+        <x:v>预期行为</x:v>
+      </x:c>
+      <x:c r="J1" s="22" t="str">
+        <x:v>业务依据/规则来源</x:v>
+      </x:c>
+      <x:c r="K1" s="22" t="str">
+        <x:v>覆盖用例 ID</x:v>
+      </x:c>
+      <x:c r="L1" s="22" t="str">
+        <x:v>覆盖状态</x:v>
+      </x:c>
+      <x:c r="M1" s="22" t="str">
+        <x:v>发现方式</x:v>
+      </x:c>
+      <x:c r="N1" s="22" t="str">
+        <x:v>素材来源</x:v>
+      </x:c>
+      <x:c r="O1" s="22" t="str">
+        <x:v>待确认问题/备注</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="84" customHeight="1">
+      <x:c r="A2" s="14" t="str">
+        <x:v>EL-LOGIN-001</x:v>
+      </x:c>
+      <x:c r="B2" s="14" t="str">
+        <x:v>STORY-001</x:v>
+      </x:c>
+      <x:c r="C2" s="14" t="str">
+        <x:v>登录页</x:v>
+      </x:c>
+      <x:c r="D2" s="14" t="str">
+        <x:v>/login</x:v>
+      </x:c>
+      <x:c r="E2" s="14" t="str">
+        <x:v>登录按钮</x:v>
+      </x:c>
+      <x:c r="F2" s="14" t="str">
+        <x:v>按钮</x:v>
+      </x:c>
+      <x:c r="G2" s="14" t="str">
+        <x:v>点击</x:v>
+      </x:c>
+      <x:c r="H2" s="14" t="str">
+        <x:v>1. 账号输入框已填写
+2. 密码输入框已填写
+3. 账号状态为启用</x:v>
+      </x:c>
+      <x:c r="I2" s="14" t="str">
+        <x:v>1. 提交登录请求
+2. 登录成功后进入工作台
+3. 登录失败时展示错误提示且不生成会话</x:v>
+      </x:c>
+      <x:c r="J2" s="14" t="str">
+        <x:v>1. 设计文档：登录主流程
+2. 验收标准：正确账号密码登录成功，错误密码登录失败
+3. 页面观察：登录页存在登录按钮</x:v>
+      </x:c>
+      <x:c r="K2" s="14" t="str">
+        <x:v>TC-LOGIN-001; TC-LOGIN-002</x:v>
+      </x:c>
+      <x:c r="L2" s="14" t="str">
+        <x:v>已覆盖</x:v>
+      </x:c>
+      <x:c r="M2" s="14" t="str">
+        <x:v>截图/浏览器实探</x:v>
+      </x:c>
+      <x:c r="N2" s="14" t="str">
+        <x:v>登录页截图、需求文档</x:v>
+      </x:c>
+      <x:c r="O2" s="14" t="str">
+        <x:v>如存在验证码或 MFA，需补充对应元素和用例</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="84" customHeight="1">
+      <x:c r="A3" s="14" t="str">
+        <x:v>EL-LOGIN-002</x:v>
+      </x:c>
+      <x:c r="B3" s="14" t="str">
+        <x:v>STORY-001</x:v>
+      </x:c>
+      <x:c r="C3" s="14" t="str">
+        <x:v>登录页</x:v>
+      </x:c>
+      <x:c r="D3" s="14" t="str">
+        <x:v>/login</x:v>
+      </x:c>
+      <x:c r="E3" s="14" t="str">
+        <x:v>忘记密码链接</x:v>
+      </x:c>
+      <x:c r="F3" s="14" t="str">
+        <x:v>链接</x:v>
+      </x:c>
+      <x:c r="G3" s="14" t="str">
+        <x:v>点击</x:v>
+      </x:c>
+      <x:c r="H3" s="14" t="str">
+        <x:v>1. 用户位于登录页
+2. 找回密码功能入口可见</x:v>
+      </x:c>
+      <x:c r="I3" s="14" t="str">
+        <x:v>1. 跳转到找回密码页面或打开找回密码流程
+2. 不应改变当前登录态</x:v>
+      </x:c>
+      <x:c r="J3" s="14" t="str">
+        <x:v>1. 页面观察：登录页存在忘记密码链接
+2. 需求文档未描述找回密码业务规则</x:v>
+      </x:c>
+      <x:c r="K3" s="14" t="str">
+        <x:v>待补充</x:v>
+      </x:c>
+      <x:c r="L3" s="14" t="str">
+        <x:v>待确认</x:v>
+      </x:c>
+      <x:c r="M3" s="14" t="str">
+        <x:v>截图</x:v>
+      </x:c>
+      <x:c r="N3" s="14" t="str">
+        <x:v>登录页截图</x:v>
+      </x:c>
+      <x:c r="O3" s="14" t="str">
+        <x:v>需确认本轮需求是否包含找回密码流程</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="8">
+    <x:dataValidation type="list" sqref="F2:F200">
+      <x:formula1>"按钮,链接,菜单,Tab,图标按钮,下拉项,输入框,上传控件,开关,复选框,单选框,表格行操作,批量操作,分页,排序,筛选,弹窗按钮,抽屉按钮,快捷入口,其他"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="G2:G200">
+      <x:formula1>"点击,双击,悬停,输入,选择,拖拽,上传,下载,快捷键,其他"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="K2:K200">
+      <x:formula1>"已覆盖,不适用,不测范围,待确认"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="L2:L200">
+      <x:formula1>"需求文档,截图,原型,浏览器实探,computer use,代码/DOM,用户说明"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="F2:F200">
+      <x:formula1>"按钮,链接,菜单,Tab,图标按钮,下拉项,输入框,上传控件,开关,复选框,单选框,表格行操作,批量操作,分页,排序,筛选,弹窗按钮,抽屉按钮,快捷入口,其他"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="G2:G200">
+      <x:formula1>"点击,双击,悬停,输入,选择,拖拽,上传,下载,快捷键,其他"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="L2:L200">
+      <x:formula1>"已覆盖,不适用,不测范围,待确认"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="M2:M200">
+      <x:formula1>"需求文档,截图,原型,浏览器实探,computer use,代码/DOM,用户说明"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3536a91d48db445e"/>
+  </x:tableParts>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Align output template with test system import format
</commit_message>
<xml_diff>
--- a/docs/test-design/codebuddy-test-design-template.xlsx
+++ b/docs/test-design/codebuddy-test-design-template.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试设计总览" sheetId="1" r:id="R9aa33bee0d574f17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求用户故事拆解" sheetId="2" r:id="R18f5be85b0144db7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试场景矩阵" sheetId="3" r:id="R1a4ee64b440c4215"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="功能测试用例" sheetId="4" r:id="R02a802871df5433f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="性能测试设计" sheetId="5" r:id="Rb4636ab274a240e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="风险与待确认问题" sheetId="6" r:id="Rd0ebf766eafd4cf2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="自动化建议" sheetId="7" r:id="R889d5606f2f34f02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面元素覆盖清单" sheetId="8" r:id="Rb1671cdb3346494e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试设计总览" sheetId="1" r:id="Rc5fd2a365a8a4ff1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求用户故事拆解" sheetId="2" r:id="Rf0e297674a5d410c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试场景矩阵" sheetId="3" r:id="Rc5df1600e1ca406e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="功能测试用例" sheetId="4" r:id="R10be33da229c4d54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="性能测试设计" sheetId="5" r:id="Rf092491958ea4770"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="风险与待确认问题" sheetId="6" r:id="R04182288200349b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="自动化建议" sheetId="7" r:id="R6f86c8492d8f4281"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面元素覆盖清单" sheetId="8" r:id="R085c75d6f08f439f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试系统导入用例" sheetId="9" r:id="R7f4564f709074c0d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -37,12 +38,17 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E79"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -80,7 +86,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="23">
+  <x:cellXfs count="27">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -134,6 +140,18 @@
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -161,6 +179,40 @@
     <x:tableColumn id="13" name="发现方式"/>
     <x:tableColumn id="14" name="素材来源"/>
     <x:tableColumn id="15" name="待确认问题/备注"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="SystemImportCasesTable" displayName="SystemImportCasesTable" ref="A1:Z2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="26">
+    <x:tableColumn id="1" name="一级模块系统编号"/>
+    <x:tableColumn id="2" name="一级模块名称"/>
+    <x:tableColumn id="3" name="二级模块系统编号"/>
+    <x:tableColumn id="4" name="二级模块名称"/>
+    <x:tableColumn id="5" name="三级模块系统编号"/>
+    <x:tableColumn id="6" name="三级模块名称"/>
+    <x:tableColumn id="7" name="四级模块系统编号"/>
+    <x:tableColumn id="8" name="四级模块名称"/>
+    <x:tableColumn id="9" name="五级模块系统编号"/>
+    <x:tableColumn id="10" name="五级模块名称"/>
+    <x:tableColumn id="11" name="其他模块系统编号"/>
+    <x:tableColumn id="12" name="其他模块名称"/>
+    <x:tableColumn id="13" name="测试用例系统编号"/>
+    <x:tableColumn id="14" name="测试用例序号"/>
+    <x:tableColumn id="15" name="测试用例名称"/>
+    <x:tableColumn id="16" name="测试步骤描述"/>
+    <x:tableColumn id="17" name="测试步骤预期结果"/>
+    <x:tableColumn id="18" name="测试类型"/>
+    <x:tableColumn id="19" name="测试用例级别"/>
+    <x:tableColumn id="20" name="执行方式"/>
+    <x:tableColumn id="21" name="测试用例说明"/>
+    <x:tableColumn id="22" name="前置条件"/>
+    <x:tableColumn id="23" name="维护人"/>
+    <x:tableColumn id="24" name="标签"/>
+    <x:tableColumn id="25" name="备注"/>
+    <x:tableColumn id="26" name="作者"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -1532,7 +1584,203 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3536a91d48db445e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ba2ddd72f0b49a8"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="14" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="32" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="42" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="42" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="18" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="18" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="18" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="36" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="36" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="18" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="18" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="18" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="26" t="str">
+        <x:v>一级模块系统编号</x:v>
+      </x:c>
+      <x:c r="B1" s="26" t="str">
+        <x:v>一级模块名称</x:v>
+      </x:c>
+      <x:c r="C1" s="26" t="str">
+        <x:v>二级模块系统编号</x:v>
+      </x:c>
+      <x:c r="D1" s="26" t="str">
+        <x:v>二级模块名称</x:v>
+      </x:c>
+      <x:c r="E1" s="26" t="str">
+        <x:v>三级模块系统编号</x:v>
+      </x:c>
+      <x:c r="F1" s="26" t="str">
+        <x:v>三级模块名称</x:v>
+      </x:c>
+      <x:c r="G1" s="26" t="str">
+        <x:v>四级模块系统编号</x:v>
+      </x:c>
+      <x:c r="H1" s="26" t="str">
+        <x:v>四级模块名称</x:v>
+      </x:c>
+      <x:c r="I1" s="26" t="str">
+        <x:v>五级模块系统编号</x:v>
+      </x:c>
+      <x:c r="J1" s="26" t="str">
+        <x:v>五级模块名称</x:v>
+      </x:c>
+      <x:c r="K1" s="26" t="str">
+        <x:v>其他模块系统编号</x:v>
+      </x:c>
+      <x:c r="L1" s="26" t="str">
+        <x:v>其他模块名称</x:v>
+      </x:c>
+      <x:c r="M1" s="26" t="str">
+        <x:v>测试用例系统编号</x:v>
+      </x:c>
+      <x:c r="N1" s="26" t="str">
+        <x:v>测试用例序号</x:v>
+      </x:c>
+      <x:c r="O1" s="26" t="str">
+        <x:v>测试用例名称</x:v>
+      </x:c>
+      <x:c r="P1" s="26" t="str">
+        <x:v>测试步骤描述</x:v>
+      </x:c>
+      <x:c r="Q1" s="26" t="str">
+        <x:v>测试步骤预期结果</x:v>
+      </x:c>
+      <x:c r="R1" s="26" t="str">
+        <x:v>测试类型</x:v>
+      </x:c>
+      <x:c r="S1" s="26" t="str">
+        <x:v>测试用例级别</x:v>
+      </x:c>
+      <x:c r="T1" s="26" t="str">
+        <x:v>执行方式</x:v>
+      </x:c>
+      <x:c r="U1" s="26" t="str">
+        <x:v>测试用例说明</x:v>
+      </x:c>
+      <x:c r="V1" s="26" t="str">
+        <x:v>前置条件</x:v>
+      </x:c>
+      <x:c r="W1" s="26" t="str">
+        <x:v>维护人</x:v>
+      </x:c>
+      <x:c r="X1" s="26" t="str">
+        <x:v>标签</x:v>
+      </x:c>
+      <x:c r="Y1" s="26" t="str">
+        <x:v>备注</x:v>
+      </x:c>
+      <x:c r="Z1" s="26" t="str">
+        <x:v>作者</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="96" customHeight="1">
+      <x:c r="A2" s="14" t="str"/>
+      <x:c r="B2" s="14" t="str">
+        <x:v>用户管理</x:v>
+      </x:c>
+      <x:c r="C2" s="14" t="str"/>
+      <x:c r="D2" s="14" t="str">
+        <x:v>用户认证</x:v>
+      </x:c>
+      <x:c r="E2" s="14" t="str"/>
+      <x:c r="F2" s="14" t="str">
+        <x:v>账号密码登录</x:v>
+      </x:c>
+      <x:c r="G2" s="14" t="str"/>
+      <x:c r="H2" s="14" t="str"/>
+      <x:c r="I2" s="14" t="str"/>
+      <x:c r="J2" s="14" t="str"/>
+      <x:c r="K2" s="14" t="str"/>
+      <x:c r="L2" s="14" t="str"/>
+      <x:c r="M2" s="14" t="str"/>
+      <x:c r="N2" s="14" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O2" s="14" t="str">
+        <x:v>正确账号密码登录成功</x:v>
+      </x:c>
+      <x:c r="P2" s="14" t="str">
+        <x:v>1. 打开登录页
+2. 输入有效账号和密码
+3. 点击登录按钮</x:v>
+      </x:c>
+      <x:c r="Q2" s="14" t="str">
+        <x:v>1. 登录成功并进入工作台
+2. 页面展示当前用户信息
+3. 系统生成有效会话</x:v>
+      </x:c>
+      <x:c r="R2" s="14" t="str">
+        <x:v>功能测试</x:v>
+      </x:c>
+      <x:c r="S2" s="14" t="str">
+        <x:v>L3</x:v>
+      </x:c>
+      <x:c r="T2" s="14" t="str">
+        <x:v>手工执行</x:v>
+      </x:c>
+      <x:c r="U2" s="14" t="str">
+        <x:v>验证账号密码登录主流程，数据来自功能测试用例 Sheet，可直接粘贴到测试系统导入模板。</x:v>
+      </x:c>
+      <x:c r="V2" s="14" t="str">
+        <x:v>1. 测试环境已部署本次需求版本
+2. 测试账号已准备且状态为启用</x:v>
+      </x:c>
+      <x:c r="W2" s="14" t="str">
+        <x:v>待填写</x:v>
+      </x:c>
+      <x:c r="X2" s="14" t="str">
+        <x:v>用户认证;登录;主流程</x:v>
+      </x:c>
+      <x:c r="Y2" s="14" t="str">
+        <x:v>该 Sheet 为测试系统导入粘贴视图，权威用例仍维护在功能测试用例 Sheet。</x:v>
+      </x:c>
+      <x:c r="Z2" s="14" t="str">
+        <x:v>待填写</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="3">
+    <x:dataValidation type="list" sqref="R2:R500">
+      <x:formula1>"功能测试,性能规格测试,可靠性测试,兼容性测试,可维护性测试,安全性测试,易用性测试"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="S2:S500">
+      <x:formula1>"L1,L2,L3,L4"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="T2:T500">
+      <x:formula1>"手工执行,自动化执行"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf724c60e439d44ee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Clarify dynamic required import fields
</commit_message>
<xml_diff>
--- a/docs/test-design/codebuddy-test-design-template.xlsx
+++ b/docs/test-design/codebuddy-test-design-template.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试设计总览" sheetId="1" r:id="Rc5fd2a365a8a4ff1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求用户故事拆解" sheetId="2" r:id="Rf0e297674a5d410c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试场景矩阵" sheetId="3" r:id="Rc5df1600e1ca406e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="功能测试用例" sheetId="4" r:id="R10be33da229c4d54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="性能测试设计" sheetId="5" r:id="Rf092491958ea4770"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="风险与待确认问题" sheetId="6" r:id="R04182288200349b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="自动化建议" sheetId="7" r:id="R6f86c8492d8f4281"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面元素覆盖清单" sheetId="8" r:id="R085c75d6f08f439f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试系统导入用例" sheetId="9" r:id="R7f4564f709074c0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试设计总览" sheetId="1" r:id="R9dc99240c3924fd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求用户故事拆解" sheetId="2" r:id="R246e5944c6054f45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试场景矩阵" sheetId="3" r:id="R15345b4737f1425d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="功能测试用例" sheetId="4" r:id="Ra1f4415195f7417d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="性能测试设计" sheetId="5" r:id="R81be98870cf842e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="风险与待确认问题" sheetId="6" r:id="R3de2c728796642be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="自动化建议" sheetId="7" r:id="Ra2304e22f59141bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面元素覆盖清单" sheetId="8" r:id="R44d17830db64463b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试系统导入用例" sheetId="9" r:id="Rabd7380a912941aa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21,7 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="3">
+  <x:fonts count="4">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -37,13 +37,24 @@
       <x:color rgb="FF1F2933"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFC00000"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E79"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -86,7 +97,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="27">
+  <x:cellXfs count="29">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -152,6 +163,12 @@
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1584,7 +1601,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ba2ddd72f0b49a8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43e1b31fdf4340b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1664,22 +1681,22 @@
       <x:c r="N1" s="26" t="str">
         <x:v>测试用例序号</x:v>
       </x:c>
-      <x:c r="O1" s="26" t="str">
+      <x:c r="O1" s="28" t="str">
         <x:v>测试用例名称</x:v>
       </x:c>
-      <x:c r="P1" s="26" t="str">
+      <x:c r="P1" s="28" t="str">
         <x:v>测试步骤描述</x:v>
       </x:c>
-      <x:c r="Q1" s="26" t="str">
+      <x:c r="Q1" s="28" t="str">
         <x:v>测试步骤预期结果</x:v>
       </x:c>
-      <x:c r="R1" s="26" t="str">
+      <x:c r="R1" s="28" t="str">
         <x:v>测试类型</x:v>
       </x:c>
-      <x:c r="S1" s="26" t="str">
+      <x:c r="S1" s="28" t="str">
         <x:v>测试用例级别</x:v>
       </x:c>
-      <x:c r="T1" s="26" t="str">
+      <x:c r="T1" s="28" t="str">
         <x:v>执行方式</x:v>
       </x:c>
       <x:c r="U1" s="26" t="str">
@@ -1780,7 +1797,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf724c60e439d44ee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b7cceeaeae74e42"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Respect system dropdown and auto fields
</commit_message>
<xml_diff>
--- a/docs/test-design/codebuddy-test-design-template.xlsx
+++ b/docs/test-design/codebuddy-test-design-template.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试设计总览" sheetId="1" r:id="R9dc99240c3924fd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求用户故事拆解" sheetId="2" r:id="R246e5944c6054f45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试场景矩阵" sheetId="3" r:id="R15345b4737f1425d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="功能测试用例" sheetId="4" r:id="Ra1f4415195f7417d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="性能测试设计" sheetId="5" r:id="R81be98870cf842e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="风险与待确认问题" sheetId="6" r:id="R3de2c728796642be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="自动化建议" sheetId="7" r:id="Ra2304e22f59141bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面元素覆盖清单" sheetId="8" r:id="R44d17830db64463b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试系统导入用例" sheetId="9" r:id="Rabd7380a912941aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试设计总览" sheetId="1" r:id="R1fdec800ca584127"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求用户故事拆解" sheetId="2" r:id="R47a4494a4d8a4929"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试场景矩阵" sheetId="3" r:id="R875844d3bcd64fa0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="功能测试用例" sheetId="4" r:id="R8f51db00d6c0491c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="性能测试设计" sheetId="5" r:id="Ra61c62b012794d30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="风险与待确认问题" sheetId="6" r:id="R200d96865b4145ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="自动化建议" sheetId="7" r:id="R7a6f11db4d9a4fca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="页面元素覆盖清单" sheetId="8" r:id="R4fdcbebd660140bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试系统导入用例" sheetId="9" r:id="Rdf90eec89d2f4b61"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1601,7 +1601,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43e1b31fdf4340b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9bf11998cbba4a24"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1761,7 +1761,7 @@
         <x:v>L3</x:v>
       </x:c>
       <x:c r="T2" s="14" t="str">
-        <x:v>手工执行</x:v>
+        <x:v>手动</x:v>
       </x:c>
       <x:c r="U2" s="14" t="str">
         <x:v>验证账号密码登录主流程，数据来自功能测试用例 Sheet，可直接粘贴到测试系统导入模板。</x:v>
@@ -1779,25 +1779,23 @@
       <x:c r="Y2" s="14" t="str">
         <x:v>该 Sheet 为测试系统导入粘贴视图，权威用例仍维护在功能测试用例 Sheet。</x:v>
       </x:c>
-      <x:c r="Z2" s="14" t="str">
-        <x:v>待填写</x:v>
-      </x:c>
+      <x:c r="Z2" s="14"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="3">
-    <x:dataValidation type="list" sqref="R2:R500">
+    <x:dataValidation type="list" allowBlank="1" sqref="R2:R500">
       <x:formula1>"功能测试,性能规格测试,可靠性测试,兼容性测试,可维护性测试,安全性测试,易用性测试"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="S2:S500">
+    <x:dataValidation type="list" allowBlank="1" sqref="S2:S500">
       <x:formula1>"L1,L2,L3,L4"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="T2:T500">
-      <x:formula1>"手工执行,自动化执行"</x:formula1>
+    <x:dataValidation type="list" allowBlank="1" sqref="T2:T500">
+      <x:formula1>"自动化,手动"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b7cceeaeae74e42"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R884dc5a6ec2d4e9b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>